<commit_message>
Simplify location input and add city color themes to export
Update location input to auto-detect US/Canada zip codes, remove country selector, and add a new "City Color Themes" sheet to the Excel export.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 0dfa28f7-9bfc-480f-943d-d4c634882f8c
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: b2dab89d-e362-4546-b0da-f06327b458d0
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/40734b85-64d2-4ba0-9dc5-6a53b140afe2/0dfa28f7-9bfc-480f-943d-d4c634882f8c/hywLa5z
</commit_message>
<xml_diff>
--- a/KnowRole_Data_Export.xlsx
+++ b/KnowRole_Data_Export.xlsx
@@ -9,7 +9,8 @@
     <sheet name="Timeout Messages" sheetId="4" r:id="rId4"/>
     <sheet name="Feedback" sheetId="5" r:id="rId5"/>
     <sheet name="Premium Questions" sheetId="6" r:id="rId6"/>
-    <sheet name="User Notes" sheetId="7" r:id="rId7"/>
+    <sheet name="City Color Themes" sheetId="7" r:id="rId7"/>
+    <sheet name="User Notes" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -14621,6 +14622,2718 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H114"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="20.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>CITY COLOR THEMES - LOCALITY SYSTEM</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>HOW THIS WORKS:</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1. User enters a US or Canada zip code</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2. App looks up the city name from zip code via zippopotam.us API</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>3. City name is matched to a team theme below</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>4. Colors are applied to accent the app design</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>EDITING NOTES:</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>- To change colors for a city, modify the Primary Color and Secondary Color columns</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>- Colors should be in hex format (e.g., #FF0000 for red)</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>- After editing, share this file back for reimport</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>City Key</v>
+      </c>
+      <c r="B14" t="str">
+        <v>City Name</v>
+      </c>
+      <c r="C14" t="str">
+        <v>State</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Major City in State</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Team Name</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Primary Color</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Secondary Color</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Accent Color</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>birmingham al</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Birmingham</v>
+      </c>
+      <c r="C15" t="str">
+        <v>AL</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Birmingham</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Crimson Tide</v>
+      </c>
+      <c r="F15" t="str">
+        <v>#9E1B32</v>
+      </c>
+      <c r="G15" t="str">
+        <v>#828A8F</v>
+      </c>
+      <c r="H15" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>huntsville</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Huntsville</v>
+      </c>
+      <c r="C16" t="str">
+        <v>AL</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Birmingham</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Crimson Tide</v>
+      </c>
+      <c r="F16" t="str">
+        <v>#9E1B32</v>
+      </c>
+      <c r="G16" t="str">
+        <v>#828A8F</v>
+      </c>
+      <c r="H16" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>fayetteville</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Fayetteville</v>
+      </c>
+      <c r="C17" t="str">
+        <v>AR</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Little Rock</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Razorbacks</v>
+      </c>
+      <c r="F17" t="str">
+        <v>#9D2235</v>
+      </c>
+      <c r="G17" t="str">
+        <v>#FFFFFF</v>
+      </c>
+      <c r="H17" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>little rock</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Little Rock</v>
+      </c>
+      <c r="C18" t="str">
+        <v>AR</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Little Rock</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Razorbacks</v>
+      </c>
+      <c r="F18" t="str">
+        <v>#9D2235</v>
+      </c>
+      <c r="G18" t="str">
+        <v>#FFFFFF</v>
+      </c>
+      <c r="H18" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>gilbert</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Gilbert</v>
+      </c>
+      <c r="C19" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Cardinals</v>
+      </c>
+      <c r="F19" t="str">
+        <v>#97233F</v>
+      </c>
+      <c r="G19" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H19" t="str">
+        <v>#FFB612</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>glendale</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Glendale</v>
+      </c>
+      <c r="C20" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Coyotes</v>
+      </c>
+      <c r="F20" t="str">
+        <v>#8C2633</v>
+      </c>
+      <c r="G20" t="str">
+        <v>#E2D6B5</v>
+      </c>
+      <c r="H20" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>mesa</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Mesa</v>
+      </c>
+      <c r="C21" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Cardinals</v>
+      </c>
+      <c r="F21" t="str">
+        <v>#97233F</v>
+      </c>
+      <c r="G21" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H21" t="str">
+        <v>#FFB612</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>phoenix</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="C22" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Cardinals</v>
+      </c>
+      <c r="F22" t="str">
+        <v>#97233F</v>
+      </c>
+      <c r="G22" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H22" t="str">
+        <v>#FFB612</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>scottsdale</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Scottsdale</v>
+      </c>
+      <c r="C23" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Suns</v>
+      </c>
+      <c r="F23" t="str">
+        <v>#1D1160</v>
+      </c>
+      <c r="G23" t="str">
+        <v>#E56020</v>
+      </c>
+      <c r="H23" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>tucson</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Tucson</v>
+      </c>
+      <c r="C24" t="str">
+        <v>AZ</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Phoenix</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Wildcats</v>
+      </c>
+      <c r="F24" t="str">
+        <v>#CC0033</v>
+      </c>
+      <c r="G24" t="str">
+        <v>#003366</v>
+      </c>
+      <c r="H24" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>anaheim</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Anaheim</v>
+      </c>
+      <c r="C25" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Ducks</v>
+      </c>
+      <c r="F25" t="str">
+        <v>#F47A38</v>
+      </c>
+      <c r="G25" t="str">
+        <v>#B9975B</v>
+      </c>
+      <c r="H25" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>bakersfield</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Bakersfield</v>
+      </c>
+      <c r="C26" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Condors</v>
+      </c>
+      <c r="F26" t="str">
+        <v>#CF4520</v>
+      </c>
+      <c r="G26" t="str">
+        <v>#003087</v>
+      </c>
+      <c r="H26" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>chula vista</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Chula Vista</v>
+      </c>
+      <c r="C27" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Padres</v>
+      </c>
+      <c r="F27" t="str">
+        <v>#2F241D</v>
+      </c>
+      <c r="G27" t="str">
+        <v>#FFC425</v>
+      </c>
+      <c r="H27" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>fontana</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Fontana</v>
+      </c>
+      <c r="C28" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Chargers</v>
+      </c>
+      <c r="F28" t="str">
+        <v>#0080C6</v>
+      </c>
+      <c r="G28" t="str">
+        <v>#FFC20E</v>
+      </c>
+      <c r="H28" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>fremont</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Fremont</v>
+      </c>
+      <c r="C29" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Warriors</v>
+      </c>
+      <c r="F29" t="str">
+        <v>#1D428A</v>
+      </c>
+      <c r="G29" t="str">
+        <v>#FFC72C</v>
+      </c>
+      <c r="H29" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>fresno</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Fresno</v>
+      </c>
+      <c r="C30" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Bulldogs</v>
+      </c>
+      <c r="F30" t="str">
+        <v>#DB0032</v>
+      </c>
+      <c r="G30" t="str">
+        <v>#002E6D</v>
+      </c>
+      <c r="H30" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>irvine</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Irvine</v>
+      </c>
+      <c r="C31" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Chargers</v>
+      </c>
+      <c r="F31" t="str">
+        <v>#0080C6</v>
+      </c>
+      <c r="G31" t="str">
+        <v>#FFC20E</v>
+      </c>
+      <c r="H31" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>los angeles</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="C32" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Rams</v>
+      </c>
+      <c r="F32" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G32" t="str">
+        <v>#FFA300</v>
+      </c>
+      <c r="H32" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>modesto</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Modesto</v>
+      </c>
+      <c r="C33" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Giants</v>
+      </c>
+      <c r="F33" t="str">
+        <v>#FD5A1E</v>
+      </c>
+      <c r="G33" t="str">
+        <v>#27251F</v>
+      </c>
+      <c r="H33" t="str">
+        <v>#EFD19F</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>moreno valley</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Moreno Valley</v>
+      </c>
+      <c r="C34" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Rams</v>
+      </c>
+      <c r="F34" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G34" t="str">
+        <v>#FFA300</v>
+      </c>
+      <c r="H34" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>oakland</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Oakland</v>
+      </c>
+      <c r="C35" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Athletics</v>
+      </c>
+      <c r="F35" t="str">
+        <v>#003831</v>
+      </c>
+      <c r="G35" t="str">
+        <v>#EFB21E</v>
+      </c>
+      <c r="H35" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>riverside</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Riverside</v>
+      </c>
+      <c r="C36" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Highlanders</v>
+      </c>
+      <c r="F36" t="str">
+        <v>#003DA5</v>
+      </c>
+      <c r="G36" t="str">
+        <v>#FFB81C</v>
+      </c>
+      <c r="H36" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>sacramento</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Sacramento</v>
+      </c>
+      <c r="C37" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Kings</v>
+      </c>
+      <c r="F37" t="str">
+        <v>#5A2D81</v>
+      </c>
+      <c r="G37" t="str">
+        <v>#63727A</v>
+      </c>
+      <c r="H37" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>san bernardino</v>
+      </c>
+      <c r="B38" t="str">
+        <v>San Bernardino</v>
+      </c>
+      <c r="C38" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Chargers</v>
+      </c>
+      <c r="F38" t="str">
+        <v>#0080C6</v>
+      </c>
+      <c r="G38" t="str">
+        <v>#FFC20E</v>
+      </c>
+      <c r="H38" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>san diego</v>
+      </c>
+      <c r="B39" t="str">
+        <v>San Diego</v>
+      </c>
+      <c r="C39" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Padres</v>
+      </c>
+      <c r="F39" t="str">
+        <v>#2F241D</v>
+      </c>
+      <c r="G39" t="str">
+        <v>#FFC425</v>
+      </c>
+      <c r="H39" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>san francisco</v>
+      </c>
+      <c r="B40" t="str">
+        <v>San Francisco</v>
+      </c>
+      <c r="C40" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E40" t="str">
+        <v>49ers</v>
+      </c>
+      <c r="F40" t="str">
+        <v>#AA0000</v>
+      </c>
+      <c r="G40" t="str">
+        <v>#B3995D</v>
+      </c>
+      <c r="H40" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>san jose</v>
+      </c>
+      <c r="B41" t="str">
+        <v>San Jose</v>
+      </c>
+      <c r="C41" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Sharks</v>
+      </c>
+      <c r="F41" t="str">
+        <v>#006D75</v>
+      </c>
+      <c r="G41" t="str">
+        <v>#EA7200</v>
+      </c>
+      <c r="H41" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>santa ana</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Santa Ana</v>
+      </c>
+      <c r="C42" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Angels</v>
+      </c>
+      <c r="F42" t="str">
+        <v>#BA0021</v>
+      </c>
+      <c r="G42" t="str">
+        <v>#003263</v>
+      </c>
+      <c r="H42" t="str">
+        <v>#C4CED4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>stockton</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Stockton</v>
+      </c>
+      <c r="C43" t="str">
+        <v>CA</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Los Angeles</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Kings</v>
+      </c>
+      <c r="F43" t="str">
+        <v>#5A2D81</v>
+      </c>
+      <c r="G43" t="str">
+        <v>#63727A</v>
+      </c>
+      <c r="H43" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>aurora</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Aurora</v>
+      </c>
+      <c r="C44" t="str">
+        <v>CO</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Denver</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Broncos</v>
+      </c>
+      <c r="F44" t="str">
+        <v>#FB4F14</v>
+      </c>
+      <c r="G44" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="H44" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>denver</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Denver</v>
+      </c>
+      <c r="C45" t="str">
+        <v>CO</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Denver</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Broncos</v>
+      </c>
+      <c r="F45" t="str">
+        <v>#FB4F14</v>
+      </c>
+      <c r="G45" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="H45" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>washington</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Washington</v>
+      </c>
+      <c r="C46" t="str">
+        <v>DC</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Washington</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Commanders</v>
+      </c>
+      <c r="F46" t="str">
+        <v>#5A1414</v>
+      </c>
+      <c r="G46" t="str">
+        <v>#FFB612</v>
+      </c>
+      <c r="H46" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>jacksonville</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Jacksonville</v>
+      </c>
+      <c r="C47" t="str">
+        <v>FL</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Jacksonville</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Jaguars</v>
+      </c>
+      <c r="F47" t="str">
+        <v>#006778</v>
+      </c>
+      <c r="G47" t="str">
+        <v>#9F792C</v>
+      </c>
+      <c r="H47" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>miami</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Miami</v>
+      </c>
+      <c r="C48" t="str">
+        <v>FL</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Jacksonville</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Dolphins</v>
+      </c>
+      <c r="F48" t="str">
+        <v>#008E97</v>
+      </c>
+      <c r="G48" t="str">
+        <v>#FC4C02</v>
+      </c>
+      <c r="H48" t="str">
+        <v>#005778</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>orlando</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Orlando</v>
+      </c>
+      <c r="C49" t="str">
+        <v>FL</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Jacksonville</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Magic</v>
+      </c>
+      <c r="F49" t="str">
+        <v>#0077C0</v>
+      </c>
+      <c r="G49" t="str">
+        <v>#C4CED4</v>
+      </c>
+      <c r="H49" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>tampa</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Tampa</v>
+      </c>
+      <c r="C50" t="str">
+        <v>FL</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Jacksonville</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Buccaneers</v>
+      </c>
+      <c r="F50" t="str">
+        <v>#D50A0A</v>
+      </c>
+      <c r="G50" t="str">
+        <v>#34302B</v>
+      </c>
+      <c r="H50" t="str">
+        <v>#FF7900</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>atlanta</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Atlanta</v>
+      </c>
+      <c r="C51" t="str">
+        <v>GA</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Atlanta</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Falcons</v>
+      </c>
+      <c r="F51" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="G51" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H51" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>des moines</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Des Moines</v>
+      </c>
+      <c r="C52" t="str">
+        <v>IA</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Des Moines</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Cyclones</v>
+      </c>
+      <c r="F52" t="str">
+        <v>#C8102E</v>
+      </c>
+      <c r="G52" t="str">
+        <v>#F1BE48</v>
+      </c>
+      <c r="H52" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>boise</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Boise</v>
+      </c>
+      <c r="C53" t="str">
+        <v>ID</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Boise</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Broncos</v>
+      </c>
+      <c r="F53" t="str">
+        <v>#0033A0</v>
+      </c>
+      <c r="G53" t="str">
+        <v>#D64309</v>
+      </c>
+      <c r="H53" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>chicago</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="C54" t="str">
+        <v>IL</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Chicago</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Bears</v>
+      </c>
+      <c r="F54" t="str">
+        <v>#0B162A</v>
+      </c>
+      <c r="G54" t="str">
+        <v>#C83803</v>
+      </c>
+      <c r="H54" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>fort wayne</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Fort Wayne</v>
+      </c>
+      <c r="C55" t="str">
+        <v>IN</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Indianapolis</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Colts</v>
+      </c>
+      <c r="F55" t="str">
+        <v>#002C5F</v>
+      </c>
+      <c r="G55" t="str">
+        <v>#A2AAAD</v>
+      </c>
+      <c r="H55" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>indianapolis</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Indianapolis</v>
+      </c>
+      <c r="C56" t="str">
+        <v>IN</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Indianapolis</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Colts</v>
+      </c>
+      <c r="F56" t="str">
+        <v>#002C5F</v>
+      </c>
+      <c r="G56" t="str">
+        <v>#A2AAAD</v>
+      </c>
+      <c r="H56" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>wichita</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Wichita</v>
+      </c>
+      <c r="C57" t="str">
+        <v>KS</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Wichita</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Shockers</v>
+      </c>
+      <c r="F57" t="str">
+        <v>#FFCD00</v>
+      </c>
+      <c r="G57" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H57" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>lexington</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Lexington</v>
+      </c>
+      <c r="C58" t="str">
+        <v>KY</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Louisville</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Wildcats</v>
+      </c>
+      <c r="F58" t="str">
+        <v>#0033A0</v>
+      </c>
+      <c r="G58" t="str">
+        <v>#FFFFFF</v>
+      </c>
+      <c r="H58" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>louisville</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Louisville</v>
+      </c>
+      <c r="C59" t="str">
+        <v>KY</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Louisville</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Cardinals</v>
+      </c>
+      <c r="F59" t="str">
+        <v>#AD0000</v>
+      </c>
+      <c r="G59" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H59" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>baton rouge</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Baton Rouge</v>
+      </c>
+      <c r="C60" t="str">
+        <v>LA</v>
+      </c>
+      <c r="D60" t="str">
+        <v>New Orleans</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Tigers</v>
+      </c>
+      <c r="F60" t="str">
+        <v>#461D7C</v>
+      </c>
+      <c r="G60" t="str">
+        <v>#FDD023</v>
+      </c>
+      <c r="H60" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>new orleans</v>
+      </c>
+      <c r="B61" t="str">
+        <v>New Orleans</v>
+      </c>
+      <c r="C61" t="str">
+        <v>LA</v>
+      </c>
+      <c r="D61" t="str">
+        <v>New Orleans</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Saints</v>
+      </c>
+      <c r="F61" t="str">
+        <v>#D3BC8D</v>
+      </c>
+      <c r="G61" t="str">
+        <v>#101820</v>
+      </c>
+      <c r="H61" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>boston</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Boston</v>
+      </c>
+      <c r="C62" t="str">
+        <v>MA</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Boston</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Patriots</v>
+      </c>
+      <c r="F62" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="G62" t="str">
+        <v>#C60C30</v>
+      </c>
+      <c r="H62" t="str">
+        <v>#B0B7BC</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>worcester</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Worcester</v>
+      </c>
+      <c r="C63" t="str">
+        <v>MA</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Boston</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Patriots</v>
+      </c>
+      <c r="F63" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="G63" t="str">
+        <v>#C60C30</v>
+      </c>
+      <c r="H63" t="str">
+        <v>#B0B7BC</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>baltimore</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Baltimore</v>
+      </c>
+      <c r="C64" t="str">
+        <v>MD</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Baltimore</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Ravens</v>
+      </c>
+      <c r="F64" t="str">
+        <v>#241773</v>
+      </c>
+      <c r="G64" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H64" t="str">
+        <v>#9E7C0C</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>detroit</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Detroit</v>
+      </c>
+      <c r="C65" t="str">
+        <v>MI</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Detroit</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Lions</v>
+      </c>
+      <c r="F65" t="str">
+        <v>#0076B6</v>
+      </c>
+      <c r="G65" t="str">
+        <v>#B0B7BC</v>
+      </c>
+      <c r="H65" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>minneapolis</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Minneapolis</v>
+      </c>
+      <c r="C66" t="str">
+        <v>MN</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Minneapolis</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Vikings</v>
+      </c>
+      <c r="F66" t="str">
+        <v>#4F2683</v>
+      </c>
+      <c r="G66" t="str">
+        <v>#FFC62F</v>
+      </c>
+      <c r="H66" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>st. paul</v>
+      </c>
+      <c r="B67" t="str">
+        <v>St. Paul</v>
+      </c>
+      <c r="C67" t="str">
+        <v>MN</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Minneapolis</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Vikings</v>
+      </c>
+      <c r="F67" t="str">
+        <v>#4F2683</v>
+      </c>
+      <c r="G67" t="str">
+        <v>#FFC62F</v>
+      </c>
+      <c r="H67" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>kansas city</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Kansas City</v>
+      </c>
+      <c r="C68" t="str">
+        <v>MO</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Kansas City</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Chiefs</v>
+      </c>
+      <c r="F68" t="str">
+        <v>#E31837</v>
+      </c>
+      <c r="G68" t="str">
+        <v>#FFB81C</v>
+      </c>
+      <c r="H68" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>st. louis</v>
+      </c>
+      <c r="B69" t="str">
+        <v>St. Louis</v>
+      </c>
+      <c r="C69" t="str">
+        <v>MO</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Kansas City</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Cardinals</v>
+      </c>
+      <c r="F69" t="str">
+        <v>#C41E3A</v>
+      </c>
+      <c r="G69" t="str">
+        <v>#0C2340</v>
+      </c>
+      <c r="H69" t="str">
+        <v>#FEDB00</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>charlotte</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Charlotte</v>
+      </c>
+      <c r="C70" t="str">
+        <v>NC</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Charlotte</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Panthers</v>
+      </c>
+      <c r="F70" t="str">
+        <v>#0085CA</v>
+      </c>
+      <c r="G70" t="str">
+        <v>#101820</v>
+      </c>
+      <c r="H70" t="str">
+        <v>#BFC0BF</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>durham</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Durham</v>
+      </c>
+      <c r="C71" t="str">
+        <v>NC</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Charlotte</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Blue Devils</v>
+      </c>
+      <c r="F71" t="str">
+        <v>#003087</v>
+      </c>
+      <c r="G71" t="str">
+        <v>#FFFFFF</v>
+      </c>
+      <c r="H71" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>greensboro</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Greensboro</v>
+      </c>
+      <c r="C72" t="str">
+        <v>NC</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Charlotte</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Panthers</v>
+      </c>
+      <c r="F72" t="str">
+        <v>#0085CA</v>
+      </c>
+      <c r="G72" t="str">
+        <v>#101820</v>
+      </c>
+      <c r="H72" t="str">
+        <v>#BFC0BF</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>raleigh</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Raleigh</v>
+      </c>
+      <c r="C73" t="str">
+        <v>NC</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Charlotte</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Hurricanes</v>
+      </c>
+      <c r="F73" t="str">
+        <v>#CC0000</v>
+      </c>
+      <c r="G73" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H73" t="str">
+        <v>#A2AAAD</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>lincoln</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Lincoln</v>
+      </c>
+      <c r="C74" t="str">
+        <v>NE</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Omaha</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Cornhuskers</v>
+      </c>
+      <c r="F74" t="str">
+        <v>#E41C38</v>
+      </c>
+      <c r="G74" t="str">
+        <v>#F5F1E7</v>
+      </c>
+      <c r="H74" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>omaha</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Omaha</v>
+      </c>
+      <c r="C75" t="str">
+        <v>NE</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Omaha</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Cornhuskers</v>
+      </c>
+      <c r="F75" t="str">
+        <v>#E41C38</v>
+      </c>
+      <c r="G75" t="str">
+        <v>#F5F1E7</v>
+      </c>
+      <c r="H75" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>jersey city</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Jersey City</v>
+      </c>
+      <c r="C76" t="str">
+        <v>NJ</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Newark</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Giants</v>
+      </c>
+      <c r="F76" t="str">
+        <v>#0B2265</v>
+      </c>
+      <c r="G76" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="H76" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>newark</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Newark</v>
+      </c>
+      <c r="C77" t="str">
+        <v>NJ</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Newark</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Devils</v>
+      </c>
+      <c r="F77" t="str">
+        <v>#CE1126</v>
+      </c>
+      <c r="G77" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H77" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>albuquerque</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Albuquerque</v>
+      </c>
+      <c r="C78" t="str">
+        <v>NM</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Albuquerque</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Lobos</v>
+      </c>
+      <c r="F78" t="str">
+        <v>#BA0C2F</v>
+      </c>
+      <c r="G78" t="str">
+        <v>#A7A8AA</v>
+      </c>
+      <c r="H78" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>las vegas</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Las Vegas</v>
+      </c>
+      <c r="C79" t="str">
+        <v>NV</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Las Vegas</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Raiders</v>
+      </c>
+      <c r="F79" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="G79" t="str">
+        <v>#A5ACAF</v>
+      </c>
+      <c r="H79" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>north las vegas</v>
+      </c>
+      <c r="B80" t="str">
+        <v>North Las Vegas</v>
+      </c>
+      <c r="C80" t="str">
+        <v>NV</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Las Vegas</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Raiders</v>
+      </c>
+      <c r="F80" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="G80" t="str">
+        <v>#A5ACAF</v>
+      </c>
+      <c r="H80" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>reno</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Reno</v>
+      </c>
+      <c r="C81" t="str">
+        <v>NV</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Las Vegas</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Wolf Pack</v>
+      </c>
+      <c r="F81" t="str">
+        <v>#003366</v>
+      </c>
+      <c r="G81" t="str">
+        <v>#807F84</v>
+      </c>
+      <c r="H81" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>brooklyn</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Brooklyn</v>
+      </c>
+      <c r="C82" t="str">
+        <v>NY</v>
+      </c>
+      <c r="D82" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Jets</v>
+      </c>
+      <c r="F82" t="str">
+        <v>#125740</v>
+      </c>
+      <c r="G82" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H82" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>buffalo</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Buffalo</v>
+      </c>
+      <c r="C83" t="str">
+        <v>NY</v>
+      </c>
+      <c r="D83" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Bills</v>
+      </c>
+      <c r="F83" t="str">
+        <v>#00338D</v>
+      </c>
+      <c r="G83" t="str">
+        <v>#C60C30</v>
+      </c>
+      <c r="H83" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>new york</v>
+      </c>
+      <c r="B84" t="str">
+        <v>New York</v>
+      </c>
+      <c r="C84" t="str">
+        <v>NY</v>
+      </c>
+      <c r="D84" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Giants</v>
+      </c>
+      <c r="F84" t="str">
+        <v>#0B2265</v>
+      </c>
+      <c r="G84" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="H84" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>rochester</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Rochester</v>
+      </c>
+      <c r="C85" t="str">
+        <v>NY</v>
+      </c>
+      <c r="D85" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Bills</v>
+      </c>
+      <c r="F85" t="str">
+        <v>#00338D</v>
+      </c>
+      <c r="G85" t="str">
+        <v>#C60C30</v>
+      </c>
+      <c r="H85" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>yonkers</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Yonkers</v>
+      </c>
+      <c r="C86" t="str">
+        <v>NY</v>
+      </c>
+      <c r="D86" t="str">
+        <v>New York</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Giants</v>
+      </c>
+      <c r="F86" t="str">
+        <v>#0B2265</v>
+      </c>
+      <c r="G86" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="H86" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>cincinnati</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Cincinnati</v>
+      </c>
+      <c r="C87" t="str">
+        <v>OH</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Columbus</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Bengals</v>
+      </c>
+      <c r="F87" t="str">
+        <v>#FB4F14</v>
+      </c>
+      <c r="G87" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H87" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>cleveland</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Cleveland</v>
+      </c>
+      <c r="C88" t="str">
+        <v>OH</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Columbus</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Browns</v>
+      </c>
+      <c r="F88" t="str">
+        <v>#311D00</v>
+      </c>
+      <c r="G88" t="str">
+        <v>#FF3C00</v>
+      </c>
+      <c r="H88" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>columbus</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Columbus</v>
+      </c>
+      <c r="C89" t="str">
+        <v>OH</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Columbus</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Blue Jackets</v>
+      </c>
+      <c r="F89" t="str">
+        <v>#002654</v>
+      </c>
+      <c r="G89" t="str">
+        <v>#CE1126</v>
+      </c>
+      <c r="H89" t="str">
+        <v>#A4A9AD</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>toledo</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Toledo</v>
+      </c>
+      <c r="C90" t="str">
+        <v>OH</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Columbus</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Rockets</v>
+      </c>
+      <c r="F90" t="str">
+        <v>#003E7E</v>
+      </c>
+      <c r="G90" t="str">
+        <v>#FFCE00</v>
+      </c>
+      <c r="H90" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>oklahoma city</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Oklahoma City</v>
+      </c>
+      <c r="C91" t="str">
+        <v>OK</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Oklahoma City</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Thunder</v>
+      </c>
+      <c r="F91" t="str">
+        <v>#007AC1</v>
+      </c>
+      <c r="G91" t="str">
+        <v>#EF3B24</v>
+      </c>
+      <c r="H91" t="str">
+        <v>#002D62</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>tulsa</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Tulsa</v>
+      </c>
+      <c r="C92" t="str">
+        <v>OK</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Oklahoma City</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Golden Hurricane</v>
+      </c>
+      <c r="F92" t="str">
+        <v>#004A8F</v>
+      </c>
+      <c r="G92" t="str">
+        <v>#C8A14F</v>
+      </c>
+      <c r="H92" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>portland</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Portland</v>
+      </c>
+      <c r="C93" t="str">
+        <v>OR</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Portland</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Trail Blazers</v>
+      </c>
+      <c r="F93" t="str">
+        <v>#E03A3E</v>
+      </c>
+      <c r="G93" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H93" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>philadelphia</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Philadelphia</v>
+      </c>
+      <c r="C94" t="str">
+        <v>PA</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Philadelphia</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Eagles</v>
+      </c>
+      <c r="F94" t="str">
+        <v>#004C54</v>
+      </c>
+      <c r="G94" t="str">
+        <v>#A5ACAF</v>
+      </c>
+      <c r="H94" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>pittsburgh</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Pittsburgh</v>
+      </c>
+      <c r="C95" t="str">
+        <v>PA</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Philadelphia</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Steelers</v>
+      </c>
+      <c r="F95" t="str">
+        <v>#FFB612</v>
+      </c>
+      <c r="G95" t="str">
+        <v>#101820</v>
+      </c>
+      <c r="H95" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>memphis</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Memphis</v>
+      </c>
+      <c r="C96" t="str">
+        <v>TN</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Nashville</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Grizzlies</v>
+      </c>
+      <c r="F96" t="str">
+        <v>#5D76A9</v>
+      </c>
+      <c r="G96" t="str">
+        <v>#12173F</v>
+      </c>
+      <c r="H96" t="str">
+        <v>#F5B112</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>nashville</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Nashville</v>
+      </c>
+      <c r="C97" t="str">
+        <v>TN</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Nashville</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Titans</v>
+      </c>
+      <c r="F97" t="str">
+        <v>#0C2340</v>
+      </c>
+      <c r="G97" t="str">
+        <v>#4B92DB</v>
+      </c>
+      <c r="H97" t="str">
+        <v>#C8102E</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>arlington</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Arlington</v>
+      </c>
+      <c r="C98" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Cowboys</v>
+      </c>
+      <c r="F98" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G98" t="str">
+        <v>#869397</v>
+      </c>
+      <c r="H98" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>austin</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Austin</v>
+      </c>
+      <c r="C99" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Longhorns</v>
+      </c>
+      <c r="F99" t="str">
+        <v>#BF5700</v>
+      </c>
+      <c r="G99" t="str">
+        <v>#333F48</v>
+      </c>
+      <c r="H99" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>dallas</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Dallas</v>
+      </c>
+      <c r="C100" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Cowboys</v>
+      </c>
+      <c r="F100" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G100" t="str">
+        <v>#869397</v>
+      </c>
+      <c r="H100" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>fort worth</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Fort Worth</v>
+      </c>
+      <c r="C101" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Cowboys</v>
+      </c>
+      <c r="F101" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G101" t="str">
+        <v>#869397</v>
+      </c>
+      <c r="H101" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>houston</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="C102" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E102" t="str">
+        <v>Texans</v>
+      </c>
+      <c r="F102" t="str">
+        <v>#03202F</v>
+      </c>
+      <c r="G102" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="H102" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>irving</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Irving</v>
+      </c>
+      <c r="C103" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E103" t="str">
+        <v>Cowboys</v>
+      </c>
+      <c r="F103" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G103" t="str">
+        <v>#869397</v>
+      </c>
+      <c r="H103" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>laredo</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Laredo</v>
+      </c>
+      <c r="C104" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E104" t="str">
+        <v>Texans</v>
+      </c>
+      <c r="F104" t="str">
+        <v>#03202F</v>
+      </c>
+      <c r="G104" t="str">
+        <v>#A71930</v>
+      </c>
+      <c r="H104" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>lubbock</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Lubbock</v>
+      </c>
+      <c r="C105" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E105" t="str">
+        <v>Red Raiders</v>
+      </c>
+      <c r="F105" t="str">
+        <v>#CC0000</v>
+      </c>
+      <c r="G105" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H105" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>plano</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Plano</v>
+      </c>
+      <c r="C106" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E106" t="str">
+        <v>Cowboys</v>
+      </c>
+      <c r="F106" t="str">
+        <v>#003594</v>
+      </c>
+      <c r="G106" t="str">
+        <v>#869397</v>
+      </c>
+      <c r="H106" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>san antonio</v>
+      </c>
+      <c r="B107" t="str">
+        <v>San Antonio</v>
+      </c>
+      <c r="C107" t="str">
+        <v>TX</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Houston</v>
+      </c>
+      <c r="E107" t="str">
+        <v>Spurs</v>
+      </c>
+      <c r="F107" t="str">
+        <v>#C4CED4</v>
+      </c>
+      <c r="G107" t="str">
+        <v>#000000</v>
+      </c>
+      <c r="H107" t="str">
+        <v>#EF426F</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>salt lake city</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Salt Lake City</v>
+      </c>
+      <c r="C108" t="str">
+        <v>UT</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Salt Lake City</v>
+      </c>
+      <c r="E108" t="str">
+        <v>Jazz</v>
+      </c>
+      <c r="F108" t="str">
+        <v>#002B5C</v>
+      </c>
+      <c r="G108" t="str">
+        <v>#F9A01B</v>
+      </c>
+      <c r="H108" t="str">
+        <v>#00471B</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>richmond</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Richmond</v>
+      </c>
+      <c r="C109" t="str">
+        <v>VA</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Virginia Beach</v>
+      </c>
+      <c r="E109" t="str">
+        <v>Commanders</v>
+      </c>
+      <c r="F109" t="str">
+        <v>#5A1414</v>
+      </c>
+      <c r="G109" t="str">
+        <v>#FFB612</v>
+      </c>
+      <c r="H109" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>seattle</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="C110" t="str">
+        <v>WA</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="E110" t="str">
+        <v>Seahawks</v>
+      </c>
+      <c r="F110" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="G110" t="str">
+        <v>#69BE28</v>
+      </c>
+      <c r="H110" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>spokane</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Spokane</v>
+      </c>
+      <c r="C111" t="str">
+        <v>WA</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="E111" t="str">
+        <v>Gonzaga</v>
+      </c>
+      <c r="F111" t="str">
+        <v>#002967</v>
+      </c>
+      <c r="G111" t="str">
+        <v>#C8102E</v>
+      </c>
+      <c r="H111" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>tacoma</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Tacoma</v>
+      </c>
+      <c r="C112" t="str">
+        <v>WA</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Seattle</v>
+      </c>
+      <c r="E112" t="str">
+        <v>Seahawks</v>
+      </c>
+      <c r="F112" t="str">
+        <v>#002244</v>
+      </c>
+      <c r="G112" t="str">
+        <v>#69BE28</v>
+      </c>
+      <c r="H112" t="str">
+        <v>#A5ACAF</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>madison</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Madison</v>
+      </c>
+      <c r="C113" t="str">
+        <v>WI</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Milwaukee</v>
+      </c>
+      <c r="E113" t="str">
+        <v>Badgers</v>
+      </c>
+      <c r="F113" t="str">
+        <v>#C5050C</v>
+      </c>
+      <c r="G113" t="str">
+        <v>#FFFFFF</v>
+      </c>
+      <c r="H113" t="str">
+        <v>#000000</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>milwaukee</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Milwaukee</v>
+      </c>
+      <c r="C114" t="str">
+        <v>WI</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Milwaukee</v>
+      </c>
+      <c r="E114" t="str">
+        <v>Packers</v>
+      </c>
+      <c r="F114" t="str">
+        <v>#203731</v>
+      </c>
+      <c r="G114" t="str">
+        <v>#FFB612</v>
+      </c>
+      <c r="H114" t="str">
+        <v>#FFFFFF</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:H114"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:A18"/>
   <cols>
     <col min="1" max="1" width="100.83203125" customWidth="1"/>

</xml_diff>